<commit_message>
Remove invalid HP & future birthdate negative test cases
</commit_message>
<xml_diff>
--- a/Tecnical test/Data Files/KaryawanBaru_Data.xlsx
+++ b/Tecnical test/Data Files/KaryawanBaru_Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -602,7 +602,6 @@
           <t>Jl. Asia Afrika No.10 Bandung</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>ktp2.jpg</t>
@@ -768,7 +767,6 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Jakarta</t>
@@ -849,7 +847,6 @@
           <t>1995-05-10</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>081234567896</t>
@@ -995,7 +992,6 @@
           <t>081234567898</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-08-15</t>
@@ -1116,7 +1112,6 @@
           <t>Jakarta</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>3201010101010010</t>
@@ -1235,212 +1230,6 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>error read ktp image file: EOF</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Test Checkbox</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Jakarta</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1995-05-10</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>3201010101010012</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>081234567812</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>a12@sv.id</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Jl. Checkbox No.6</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>ktp11.jpg</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>selfie12.jpg</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Test HP Non-Angka</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Jakarta</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>1995-05-10</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>3201010101010013</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>abc123</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>a13@sv.id</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Jl. H No.8</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Jl. H No.8</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>ktp12.jpg</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>selfie12.jpg</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Format nomor HP tidak valid</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Test Tgl Lahir Depan</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Jakarta</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2030-01-01</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>3201010101010014</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>081234567814</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>a14@sv.id</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Jl. I No.9</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Jl. I No.9</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>ktp1.jpg</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>selfie1.jpg</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Tanggal lahir tidak boleh di masa depan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore Test Checkbox row in karyawan baru test data
</commit_message>
<xml_diff>
--- a/Tecnical test/Data Files/KaryawanBaru_Data.xlsx
+++ b/Tecnical test/Data Files/KaryawanBaru_Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1230,6 +1230,71 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>error read ktp image file: EOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Test Checkbox</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jakarta</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1995-05-10</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3201010101010012</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>081234567812</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>a12@sv.id</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Jl. Checkbox No.6</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ktp11.jpg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>selfie12.jpg</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
     </row>

</xml_diff>